<commit_message>
excel formula bug fixed
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77F30D6-0A61-714F-A908-1B495323CF66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FE70A3-F838-6745-A36B-52FF9603505B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataType Dropdown Items" sheetId="1" state="hidden" r:id="rId1"/>
@@ -91,9 +91,10 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
@@ -104,6 +105,20 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </cellMetadata>
   <valueMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
@@ -3786,7 +3801,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="39.1640625" bestFit="1" customWidth="1"/>
@@ -3850,8 +3865,8 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="113" t="e" vm="1">
-        <f t="array" ref="A6:A17">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Table7[Table Name], Table7[Table Name]&lt;&gt;""))</f>
+      <c r="A6" s="113" t="e" cm="1" vm="1">
+        <f t="array" ref="A6">_xlfn.UNIQUE(_xlfn._xlws.FILTER(Table7[Table Name], Table7[Table Name]&lt;&gt;""))</f>
         <v>#VALUE!</v>
       </c>
       <c r="B6" s="114"/>
@@ -3860,99 +3875,77 @@
       <c r="E6" s="115"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A7" s="116"/>
       <c r="B7" s="117"/>
       <c r="C7" s="117"/>
       <c r="D7" s="117"/>
       <c r="E7" s="118"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A8" s="113"/>
       <c r="B8" s="114"/>
       <c r="C8" s="114"/>
       <c r="D8" s="114"/>
       <c r="E8" s="115"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A9" s="116"/>
       <c r="B9" s="117"/>
       <c r="C9" s="117"/>
       <c r="D9" s="117"/>
       <c r="E9" s="118"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A10" s="113"/>
       <c r="B10" s="114"/>
       <c r="C10" s="114"/>
       <c r="D10" s="114"/>
       <c r="E10" s="115"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A11" s="116"/>
       <c r="B11" s="117"/>
       <c r="C11" s="117"/>
       <c r="D11" s="117"/>
       <c r="E11" s="118"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A12" s="113"/>
       <c r="B12" s="114"/>
       <c r="C12" s="114"/>
       <c r="D12" s="114"/>
       <c r="E12" s="115"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A13" s="116"/>
       <c r="B13" s="117"/>
       <c r="C13" s="117"/>
       <c r="D13" s="117"/>
       <c r="E13" s="118"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A14" s="113"/>
       <c r="B14" s="114"/>
       <c r="C14" s="114"/>
       <c r="D14" s="114"/>
       <c r="E14" s="115"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A15" s="116"/>
       <c r="B15" s="117"/>
       <c r="C15" s="117"/>
       <c r="D15" s="117"/>
       <c r="E15" s="118"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="113" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A16" s="113"/>
       <c r="B16" s="114"/>
       <c r="C16" s="114"/>
       <c r="D16" s="114"/>
       <c r="E16" s="115"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="116" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
+      <c r="A17" s="116"/>
       <c r="B17" s="117"/>
       <c r="C17" s="117"/>
       <c r="D17" s="117"/>
@@ -4034,6 +4027,510 @@
       <c r="C28" s="108"/>
       <c r="D28" s="108"/>
       <c r="E28" s="109"/>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="116"/>
+      <c r="B29" s="117"/>
+      <c r="C29" s="117"/>
+      <c r="D29" s="117"/>
+      <c r="E29" s="118"/>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="119"/>
+      <c r="B30" s="108"/>
+      <c r="C30" s="108"/>
+      <c r="D30" s="108"/>
+      <c r="E30" s="109"/>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="116"/>
+      <c r="B31" s="117"/>
+      <c r="C31" s="117"/>
+      <c r="D31" s="117"/>
+      <c r="E31" s="118"/>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="119"/>
+      <c r="B32" s="108"/>
+      <c r="C32" s="108"/>
+      <c r="D32" s="108"/>
+      <c r="E32" s="109"/>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="116"/>
+      <c r="B33" s="117"/>
+      <c r="C33" s="117"/>
+      <c r="D33" s="117"/>
+      <c r="E33" s="118"/>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="119"/>
+      <c r="B34" s="108"/>
+      <c r="C34" s="108"/>
+      <c r="D34" s="108"/>
+      <c r="E34" s="109"/>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="116"/>
+      <c r="B35" s="117"/>
+      <c r="C35" s="117"/>
+      <c r="D35" s="117"/>
+      <c r="E35" s="118"/>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="119"/>
+      <c r="B36" s="108"/>
+      <c r="C36" s="108"/>
+      <c r="D36" s="108"/>
+      <c r="E36" s="109"/>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="116"/>
+      <c r="B37" s="117"/>
+      <c r="C37" s="117"/>
+      <c r="D37" s="117"/>
+      <c r="E37" s="118"/>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="119"/>
+      <c r="B38" s="108"/>
+      <c r="C38" s="108"/>
+      <c r="D38" s="108"/>
+      <c r="E38" s="109"/>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="116"/>
+      <c r="B39" s="117"/>
+      <c r="C39" s="117"/>
+      <c r="D39" s="117"/>
+      <c r="E39" s="118"/>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="119"/>
+      <c r="B40" s="108"/>
+      <c r="C40" s="108"/>
+      <c r="D40" s="108"/>
+      <c r="E40" s="109"/>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="116"/>
+      <c r="B41" s="117"/>
+      <c r="C41" s="117"/>
+      <c r="D41" s="117"/>
+      <c r="E41" s="118"/>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="119"/>
+      <c r="B42" s="108"/>
+      <c r="C42" s="108"/>
+      <c r="D42" s="108"/>
+      <c r="E42" s="109"/>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="116"/>
+      <c r="B43" s="117"/>
+      <c r="C43" s="117"/>
+      <c r="D43" s="117"/>
+      <c r="E43" s="118"/>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="119"/>
+      <c r="B44" s="108"/>
+      <c r="C44" s="108"/>
+      <c r="D44" s="108"/>
+      <c r="E44" s="109"/>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="116"/>
+      <c r="B45" s="117"/>
+      <c r="C45" s="117"/>
+      <c r="D45" s="117"/>
+      <c r="E45" s="118"/>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="119"/>
+      <c r="B46" s="108"/>
+      <c r="C46" s="108"/>
+      <c r="D46" s="108"/>
+      <c r="E46" s="109"/>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="116"/>
+      <c r="B47" s="117"/>
+      <c r="C47" s="117"/>
+      <c r="D47" s="117"/>
+      <c r="E47" s="118"/>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="119"/>
+      <c r="B48" s="108"/>
+      <c r="C48" s="108"/>
+      <c r="D48" s="108"/>
+      <c r="E48" s="109"/>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" s="116"/>
+      <c r="B49" s="117"/>
+      <c r="C49" s="117"/>
+      <c r="D49" s="117"/>
+      <c r="E49" s="118"/>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="119"/>
+      <c r="B50" s="108"/>
+      <c r="C50" s="108"/>
+      <c r="D50" s="108"/>
+      <c r="E50" s="109"/>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" s="116"/>
+      <c r="B51" s="117"/>
+      <c r="C51" s="117"/>
+      <c r="D51" s="117"/>
+      <c r="E51" s="118"/>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" s="119"/>
+      <c r="B52" s="108"/>
+      <c r="C52" s="108"/>
+      <c r="D52" s="108"/>
+      <c r="E52" s="109"/>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" s="116"/>
+      <c r="B53" s="117"/>
+      <c r="C53" s="117"/>
+      <c r="D53" s="117"/>
+      <c r="E53" s="118"/>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" s="119"/>
+      <c r="B54" s="108"/>
+      <c r="C54" s="108"/>
+      <c r="D54" s="108"/>
+      <c r="E54" s="109"/>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" s="116"/>
+      <c r="B55" s="117"/>
+      <c r="C55" s="117"/>
+      <c r="D55" s="117"/>
+      <c r="E55" s="118"/>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" s="119"/>
+      <c r="B56" s="108"/>
+      <c r="C56" s="108"/>
+      <c r="D56" s="108"/>
+      <c r="E56" s="109"/>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" s="116"/>
+      <c r="B57" s="117"/>
+      <c r="C57" s="117"/>
+      <c r="D57" s="117"/>
+      <c r="E57" s="118"/>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" s="119"/>
+      <c r="B58" s="108"/>
+      <c r="C58" s="108"/>
+      <c r="D58" s="108"/>
+      <c r="E58" s="109"/>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" s="116"/>
+      <c r="B59" s="117"/>
+      <c r="C59" s="117"/>
+      <c r="D59" s="117"/>
+      <c r="E59" s="118"/>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" s="119"/>
+      <c r="B60" s="108"/>
+      <c r="C60" s="108"/>
+      <c r="D60" s="108"/>
+      <c r="E60" s="109"/>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" s="116"/>
+      <c r="B61" s="117"/>
+      <c r="C61" s="117"/>
+      <c r="D61" s="117"/>
+      <c r="E61" s="118"/>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" s="119"/>
+      <c r="B62" s="108"/>
+      <c r="C62" s="108"/>
+      <c r="D62" s="108"/>
+      <c r="E62" s="109"/>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" s="116"/>
+      <c r="B63" s="117"/>
+      <c r="C63" s="117"/>
+      <c r="D63" s="117"/>
+      <c r="E63" s="118"/>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" s="119"/>
+      <c r="B64" s="108"/>
+      <c r="C64" s="108"/>
+      <c r="D64" s="108"/>
+      <c r="E64" s="109"/>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" s="116"/>
+      <c r="B65" s="117"/>
+      <c r="C65" s="117"/>
+      <c r="D65" s="117"/>
+      <c r="E65" s="118"/>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="119"/>
+      <c r="B66" s="108"/>
+      <c r="C66" s="108"/>
+      <c r="D66" s="108"/>
+      <c r="E66" s="109"/>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="116"/>
+      <c r="B67" s="117"/>
+      <c r="C67" s="117"/>
+      <c r="D67" s="117"/>
+      <c r="E67" s="118"/>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="119"/>
+      <c r="B68" s="108"/>
+      <c r="C68" s="108"/>
+      <c r="D68" s="108"/>
+      <c r="E68" s="109"/>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="116"/>
+      <c r="B69" s="117"/>
+      <c r="C69" s="117"/>
+      <c r="D69" s="117"/>
+      <c r="E69" s="118"/>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="119"/>
+      <c r="B70" s="108"/>
+      <c r="C70" s="108"/>
+      <c r="D70" s="108"/>
+      <c r="E70" s="109"/>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="116"/>
+      <c r="B71" s="117"/>
+      <c r="C71" s="117"/>
+      <c r="D71" s="117"/>
+      <c r="E71" s="118"/>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="119"/>
+      <c r="B72" s="108"/>
+      <c r="C72" s="108"/>
+      <c r="D72" s="108"/>
+      <c r="E72" s="109"/>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="116"/>
+      <c r="B73" s="117"/>
+      <c r="C73" s="117"/>
+      <c r="D73" s="117"/>
+      <c r="E73" s="118"/>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="119"/>
+      <c r="B74" s="108"/>
+      <c r="C74" s="108"/>
+      <c r="D74" s="108"/>
+      <c r="E74" s="109"/>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="116"/>
+      <c r="B75" s="117"/>
+      <c r="C75" s="117"/>
+      <c r="D75" s="117"/>
+      <c r="E75" s="118"/>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="119"/>
+      <c r="B76" s="108"/>
+      <c r="C76" s="108"/>
+      <c r="D76" s="108"/>
+      <c r="E76" s="109"/>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="116"/>
+      <c r="B77" s="117"/>
+      <c r="C77" s="117"/>
+      <c r="D77" s="117"/>
+      <c r="E77" s="118"/>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="119"/>
+      <c r="B78" s="108"/>
+      <c r="C78" s="108"/>
+      <c r="D78" s="108"/>
+      <c r="E78" s="109"/>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="116"/>
+      <c r="B79" s="117"/>
+      <c r="C79" s="117"/>
+      <c r="D79" s="117"/>
+      <c r="E79" s="118"/>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" s="119"/>
+      <c r="B80" s="108"/>
+      <c r="C80" s="108"/>
+      <c r="D80" s="108"/>
+      <c r="E80" s="109"/>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="116"/>
+      <c r="B81" s="117"/>
+      <c r="C81" s="117"/>
+      <c r="D81" s="117"/>
+      <c r="E81" s="118"/>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="119"/>
+      <c r="B82" s="108"/>
+      <c r="C82" s="108"/>
+      <c r="D82" s="108"/>
+      <c r="E82" s="109"/>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" s="116"/>
+      <c r="B83" s="117"/>
+      <c r="C83" s="117"/>
+      <c r="D83" s="117"/>
+      <c r="E83" s="118"/>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="119"/>
+      <c r="B84" s="108"/>
+      <c r="C84" s="108"/>
+      <c r="D84" s="108"/>
+      <c r="E84" s="109"/>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="116"/>
+      <c r="B85" s="117"/>
+      <c r="C85" s="117"/>
+      <c r="D85" s="117"/>
+      <c r="E85" s="118"/>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="119"/>
+      <c r="B86" s="108"/>
+      <c r="C86" s="108"/>
+      <c r="D86" s="108"/>
+      <c r="E86" s="109"/>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="116"/>
+      <c r="B87" s="117"/>
+      <c r="C87" s="117"/>
+      <c r="D87" s="117"/>
+      <c r="E87" s="118"/>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" s="119"/>
+      <c r="B88" s="108"/>
+      <c r="C88" s="108"/>
+      <c r="D88" s="108"/>
+      <c r="E88" s="109"/>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" s="116"/>
+      <c r="B89" s="117"/>
+      <c r="C89" s="117"/>
+      <c r="D89" s="117"/>
+      <c r="E89" s="118"/>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" s="119"/>
+      <c r="B90" s="108"/>
+      <c r="C90" s="108"/>
+      <c r="D90" s="108"/>
+      <c r="E90" s="109"/>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" s="116"/>
+      <c r="B91" s="117"/>
+      <c r="C91" s="117"/>
+      <c r="D91" s="117"/>
+      <c r="E91" s="118"/>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92" s="119"/>
+      <c r="B92" s="108"/>
+      <c r="C92" s="108"/>
+      <c r="D92" s="108"/>
+      <c r="E92" s="109"/>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93" s="116"/>
+      <c r="B93" s="117"/>
+      <c r="C93" s="117"/>
+      <c r="D93" s="117"/>
+      <c r="E93" s="118"/>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94" s="119"/>
+      <c r="B94" s="108"/>
+      <c r="C94" s="108"/>
+      <c r="D94" s="108"/>
+      <c r="E94" s="109"/>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95" s="116"/>
+      <c r="B95" s="117"/>
+      <c r="C95" s="117"/>
+      <c r="D95" s="117"/>
+      <c r="E95" s="118"/>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96" s="119"/>
+      <c r="B96" s="108"/>
+      <c r="C96" s="108"/>
+      <c r="D96" s="108"/>
+      <c r="E96" s="109"/>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97" s="116"/>
+      <c r="B97" s="117"/>
+      <c r="C97" s="117"/>
+      <c r="D97" s="117"/>
+      <c r="E97" s="118"/>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98" s="119"/>
+      <c r="B98" s="108"/>
+      <c r="C98" s="108"/>
+      <c r="D98" s="108"/>
+      <c r="E98" s="109"/>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99" s="116"/>
+      <c r="B99" s="117"/>
+      <c r="C99" s="117"/>
+      <c r="D99" s="117"/>
+      <c r="E99" s="118"/>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100" s="119"/>
+      <c r="B100" s="108"/>
+      <c r="C100" s="108"/>
+      <c r="D100" s="108"/>
+      <c r="E100" s="109"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Null related bugs fixed
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94FE70A3-F838-6745-A36B-52FF9603505B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F5F388-2749-614C-B54C-731A88DEF297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataType Dropdown Items" sheetId="1" state="hidden" r:id="rId1"/>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="213">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -2889,6 +2889,69 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="center"/>
     </dxf>
     <dxf>
@@ -2911,69 +2974,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="bottom"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -3083,32 +3083,32 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="124" dataDxfId="123">
   <autoFilter ref="A3:D4" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="110"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="119"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="124">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="118">
   <autoFilter ref="A5:H28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="123">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="117">
       <calculatedColumnFormula>ROW()-5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="121"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="119"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="118"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="117"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="116"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="115"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="114"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="113"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="112"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="111"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="110"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5340,7 +5340,9 @@
       <c r="E27" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="F27" s="27"/>
+      <c r="F27" s="27" t="s">
+        <v>130</v>
+      </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
     </row>
@@ -5361,7 +5363,9 @@
       <c r="E28" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="F28" s="4"/>
+      <c r="F28" s="27" t="s">
+        <v>130</v>
+      </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
     </row>

</xml_diff>

<commit_message>
SystemCommon: Optimistic Locking dataType removed
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49F5F388-2749-614C-B54C-731A88DEF297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2057154-E648-4847-8700-384C58EE8FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="213">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -2889,6 +2889,30 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="center"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill>
           <bgColor auto="1"/>
@@ -2950,30 +2974,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="center"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -3083,32 +3083,32 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="124" dataDxfId="123">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table5" displayName="Table5" ref="A3:D4" totalsRowShown="0" headerRowDxfId="115" dataDxfId="114">
   <autoFilter ref="A3:D4" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="121"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="119"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Date" dataDxfId="113"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Version" dataDxfId="112"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Changes" dataDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Changed By" dataDxfId="110"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="118">
-  <autoFilter ref="A5:H28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H27" totalsRowShown="0" dataDxfId="124">
+  <autoFilter ref="A5:H27" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="117">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="123">
       <calculatedColumnFormula>ROW()-5</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="116"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="115"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="114"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="113"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="112"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="111"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="110"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Category" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Category Name" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Key" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Description" dataDxfId="119"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Required" dataDxfId="118"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Value" dataDxfId="117"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Notes" dataDxfId="116"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4819,7 +4819,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.5" bestFit="1" customWidth="1"/>
@@ -4870,7 +4870,7 @@
     </row>
     <row r="6" spans="1:8" ht="16" customHeight="1">
       <c r="A6" s="1">
-        <f t="shared" ref="A6:A28" si="0">ROW()-5</f>
+        <f t="shared" ref="A6:A27" si="0">ROW()-5</f>
         <v>1</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -5345,29 +5345,6 @@
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
-    </row>
-    <row r="28" spans="1:8" ht="16" customHeight="1">
-      <c r="A28" s="1">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="F28" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Default values added to GeneralSettings sheet
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2057154-E648-4847-8700-384C58EE8FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD44E2CA-420A-1C41-A820-14AC0A1BFF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="216">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -793,6 +793,15 @@
   </si>
   <si>
     <t>Table Display Name (Additional Lang 3)</t>
+  </si>
+  <si>
+    <t>VERSION</t>
+  </si>
+  <si>
+    <t>UTF-8</t>
+  </si>
+  <si>
+    <t>en</t>
   </si>
 </sst>
 </file>
@@ -3832,7 +3841,7 @@
     <row r="3" spans="1:5">
       <c r="B3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
-        <v/>
+        <v>en</v>
       </c>
       <c r="C3" s="32" t="str">
         <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
@@ -4959,7 +4968,9 @@
       <c r="F9" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="H9" s="1"/>
     </row>
     <row r="10" spans="1:8" ht="16" customHeight="1">
@@ -4982,7 +4993,9 @@
       <c r="F10" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1" t="s">
+        <v>214</v>
+      </c>
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="1:8" ht="32" customHeight="1">
@@ -5005,7 +5018,9 @@
       <c r="F11" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G11" s="1"/>
+      <c r="G11" s="1" t="s">
+        <v>215</v>
+      </c>
       <c r="H11" s="1"/>
     </row>
     <row r="12" spans="1:8" ht="48" customHeight="1">
@@ -5343,7 +5358,9 @@
       <c r="F27" s="27" t="s">
         <v>130</v>
       </c>
-      <c r="G27" s="1"/>
+      <c r="G27" s="1" t="s">
+        <v>213</v>
+      </c>
       <c r="H27" s="1"/>
     </row>
   </sheetData>
@@ -5415,7 +5432,7 @@
       <c r="B3" s="3"/>
       <c r="P3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
-        <v/>
+        <v>en</v>
       </c>
       <c r="Q3" s="32" t="str">
         <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
@@ -6529,7 +6546,7 @@
       <c r="D4" s="52"/>
       <c r="F4" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
-        <v/>
+        <v>en</v>
       </c>
       <c r="G4" s="32" t="str">
         <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
@@ -6932,7 +6949,7 @@
       <c r="A3" s="52"/>
       <c r="AH3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
-        <v/>
+        <v>en</v>
       </c>
       <c r="AI3" s="32" t="str">
         <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>
@@ -10727,7 +10744,7 @@
       <c r="A3" s="52"/>
       <c r="AH3" s="32" t="str">
         <f>IF('General Settings'!$G$11=0,"",'General Settings'!$G$11)</f>
-        <v/>
+        <v>en</v>
       </c>
       <c r="AI3" s="32" t="str">
         <f>IF('General Settings'!$G$12=0,"",'General Settings'!$G$12)</f>

</xml_diff>

<commit_message>
Optimistic Locking - dataType column item recovered
</commit_message>
<xml_diff>
--- a/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
+++ b/excel-format/db-column-definitions_fmt-v5.0.0-en_my-app.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yosuke.tanaka/Desktop/development/git/ecuacion-tool-code-generator/excel-format/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD44E2CA-420A-1C41-A820-14AC0A1BFF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46F3CBA-1473-4246-9034-2C7E81A23414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="11700" tabRatio="853" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="216">
   <si>
     <t>DB Common Item Definition</t>
   </si>
@@ -3105,8 +3105,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H27" totalsRowShown="0" dataDxfId="124">
-  <autoFilter ref="A5:H27" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table50" displayName="Table50" ref="A5:H28" totalsRowShown="0" dataDxfId="124">
+  <autoFilter ref="A5:H28" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="#" dataDxfId="123">
       <calculatedColumnFormula>ROW()-5</calculatedColumnFormula>
@@ -4828,7 +4828,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.5" bestFit="1" customWidth="1"/>
@@ -5362,6 +5362,29 @@
         <v>213</v>
       </c>
       <c r="H27" s="1"/>
+    </row>
+    <row r="28" spans="1:8" ht="16">
+      <c r="A28" s="1">
+        <f>ROW()-5</f>
+        <v>23</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>